<commit_message>
al-nisa correction 10 - 20
</commit_message>
<xml_diff>
--- a/verification_detailed.xlsx
+++ b/verification_detailed.xlsx
@@ -25368,13 +25368,13 @@
         <v>122</v>
       </c>
       <c r="E892" t="n">
-        <v>6083</v>
+        <v>6194</v>
       </c>
       <c r="F892" t="n">
-        <v>2240</v>
+        <v>2350</v>
       </c>
       <c r="G892" t="n">
-        <v>3843</v>
+        <v>3844</v>
       </c>
     </row>
     <row r="893">
@@ -25426,13 +25426,13 @@
         <v>124</v>
       </c>
       <c r="E894" t="n">
-        <v>6071</v>
+        <v>6182</v>
       </c>
       <c r="F894" t="n">
-        <v>2339</v>
+        <v>2449</v>
       </c>
       <c r="G894" t="n">
-        <v>3732</v>
+        <v>3733</v>
       </c>
     </row>
     <row r="895">
@@ -25455,13 +25455,13 @@
         <v>125</v>
       </c>
       <c r="E895" t="n">
-        <v>7337</v>
+        <v>7448</v>
       </c>
       <c r="F895" t="n">
-        <v>2402</v>
+        <v>2512</v>
       </c>
       <c r="G895" t="n">
-        <v>4935</v>
+        <v>4936</v>
       </c>
     </row>
     <row r="896">
@@ -26064,13 +26064,13 @@
         <v>146</v>
       </c>
       <c r="E916" t="n">
-        <v>7995</v>
+        <v>8106</v>
       </c>
       <c r="F916" t="n">
-        <v>3391</v>
+        <v>3501</v>
       </c>
       <c r="G916" t="n">
-        <v>4604</v>
+        <v>4605</v>
       </c>
     </row>
     <row r="917">
@@ -27657,13 +27657,13 @@
       </c>
       <c r="D971" s="3" t="inlineStr"/>
       <c r="E971" s="3" t="n">
-        <v>1673548</v>
+        <v>1673992</v>
       </c>
       <c r="F971" s="3" t="n">
-        <v>617782</v>
+        <v>618222</v>
       </c>
       <c r="G971" s="3" t="n">
-        <v>1055766</v>
+        <v>1055770</v>
       </c>
     </row>
     <row r="972">
@@ -28005,13 +28005,13 @@
         <v>11</v>
       </c>
       <c r="E984" t="n">
-        <v>27891</v>
+        <v>27780</v>
       </c>
       <c r="F984" t="n">
-        <v>11571</v>
+        <v>11461</v>
       </c>
       <c r="G984" t="n">
-        <v>16320</v>
+        <v>16319</v>
       </c>
     </row>
     <row r="985">
@@ -32817,13 +32817,13 @@
       </c>
       <c r="D1150" s="3" t="inlineStr"/>
       <c r="E1150" s="3" t="n">
-        <v>1706227</v>
+        <v>1706116</v>
       </c>
       <c r="F1150" s="3" t="n">
-        <v>645984</v>
+        <v>645874</v>
       </c>
       <c r="G1150" s="3" t="n">
-        <v>1060243</v>
+        <v>1060242</v>
       </c>
     </row>
     <row r="1151">

</xml_diff>